<commit_message>
Update backup proposal log data with latest entries
Update backup file `proposal-log-2026-04-11.xlsx` to reflect current state.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: b8c342de-3a7a-4a8d-b4a3-2df3949c2128
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: fc16eac6-f6b1-4767-bb00-01c40a09fe58
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/f7cd70f1-dedb-4f27-8c85-9633fe48f13e/b8c342de-3a7a-4a8d-b4a3-2df3949c2128/Gvtrz9L
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/backups/proposal-log-2026-04-11.xlsx
+++ b/backups/proposal-log-2026-04-11.xlsx
@@ -382,21 +382,33 @@
     <t>JW</t>
   </si>
   <si>
+    <t>26-0205</t>
+  </si>
+  <si>
+    <t>TRA General Office Complex</t>
+  </si>
+  <si>
+    <t>2026-04-02</t>
+  </si>
+  <si>
+    <t>2026-04-23</t>
+  </si>
+  <si>
+    <t>Won</t>
+  </si>
+  <si>
+    <t>2026-08-03</t>
+  </si>
+  <si>
+    <t>2027-07-30</t>
+  </si>
+  <si>
     <t>26-0213</t>
   </si>
   <si>
-    <t>TRA General Office Complex</t>
-  </si>
-  <si>
     <t>DFW</t>
   </si>
   <si>
-    <t>2026-04-02</t>
-  </si>
-  <si>
-    <t>2026-04-23</t>
-  </si>
-  <si>
     <t>Christman Weeks</t>
   </si>
   <si>
@@ -406,18 +418,6 @@
     <t>["69ce6ad9ffa00f5f6b96a4d9"]</t>
   </si>
   <si>
-    <t>26-0205</t>
-  </si>
-  <si>
-    <t>Won</t>
-  </si>
-  <si>
-    <t>2026-08-03</t>
-  </si>
-  <si>
-    <t>2027-07-30</t>
-  </si>
-  <si>
     <t>26-0211</t>
   </si>
   <si>
@@ -793,6 +793,39 @@
     <t>2028-02-01</t>
   </si>
   <si>
+    <t>26-0020</t>
+  </si>
+  <si>
+    <t>26-0196</t>
+  </si>
+  <si>
+    <t>Univ of Oregon - Esslinger Hall Re-roof</t>
+  </si>
+  <si>
+    <t>2026-03-24</t>
+  </si>
+  <si>
+    <t>2026-04-07</t>
+  </si>
+  <si>
+    <t>Mark Socks</t>
+  </si>
+  <si>
+    <t>Lost</t>
+  </si>
+  <si>
+    <t>NO BID - No Scope</t>
+  </si>
+  <si>
+    <t>https://app.buildingconnected.com/opportunities/69c1b75e4cb9ae021994a5b7</t>
+  </si>
+  <si>
+    <t>["69c1b75e4cb9ae021994a5b7"]</t>
+  </si>
+  <si>
+    <t>["Expansion Control Systems"]</t>
+  </si>
+  <si>
     <t>26-0194</t>
   </si>
   <si>
@@ -817,7 +850,28 @@
     <t>QA Reviewer</t>
   </si>
   <si>
-    <t>26-0020</t>
+    <t>26-0200</t>
+  </si>
+  <si>
+    <t>Flying Pickle Idaho Falls</t>
+  </si>
+  <si>
+    <t>Washington (SEA)</t>
+  </si>
+  <si>
+    <t>2026-03-31</t>
+  </si>
+  <si>
+    <t>Jake Marrujo</t>
+  </si>
+  <si>
+    <t>https://app.buildingconnected.com/opportunities/69cc01834e68f2d35d122b59</t>
+  </si>
+  <si>
+    <t>["69cc01834e68f2d35d122b59"]</t>
+  </si>
+  <si>
+    <t>[]</t>
   </si>
   <si>
     <t>26-0214</t>
@@ -847,60 +901,6 @@
     <t>["2026-04-08T18:09:51.975Z: dueDate: 2026-04-07 → 2026-04-13"]</t>
   </si>
   <si>
-    <t>26-0200</t>
-  </si>
-  <si>
-    <t>Flying Pickle Idaho Falls</t>
-  </si>
-  <si>
-    <t>Washington (SEA)</t>
-  </si>
-  <si>
-    <t>2026-03-31</t>
-  </si>
-  <si>
-    <t>Jake Marrujo</t>
-  </si>
-  <si>
-    <t>https://app.buildingconnected.com/opportunities/69cc01834e68f2d35d122b59</t>
-  </si>
-  <si>
-    <t>["69cc01834e68f2d35d122b59"]</t>
-  </si>
-  <si>
-    <t>[]</t>
-  </si>
-  <si>
-    <t>26-0196</t>
-  </si>
-  <si>
-    <t>Univ of Oregon - Esslinger Hall Re-roof</t>
-  </si>
-  <si>
-    <t>2026-03-24</t>
-  </si>
-  <si>
-    <t>2026-04-07</t>
-  </si>
-  <si>
-    <t>Mark Socks</t>
-  </si>
-  <si>
-    <t>Lost</t>
-  </si>
-  <si>
-    <t>NO BID - No Scope</t>
-  </si>
-  <si>
-    <t>https://app.buildingconnected.com/opportunities/69c1b75e4cb9ae021994a5b7</t>
-  </si>
-  <si>
-    <t>["69c1b75e4cb9ae021994a5b7"]</t>
-  </si>
-  <si>
-    <t>["Expansion Control Systems"]</t>
-  </si>
-  <si>
     <t>26-0003</t>
   </si>
   <si>
@@ -1042,6 +1042,57 @@
     <t>1057256</t>
   </si>
   <si>
+    <t>ATL - Atlanta</t>
+  </si>
+  <si>
+    <t>Declined</t>
+  </si>
+  <si>
+    <t>Joey Dinelli</t>
+  </si>
+  <si>
+    <t>["2026-04-02T22:49:34.183Z: Rejected by Haley Kruse"]</t>
+  </si>
+  <si>
+    <t>26-0195</t>
+  </si>
+  <si>
+    <t>2026-03-26</t>
+  </si>
+  <si>
+    <t>https://app.buildingconnected.com/opportunities/69c161e5eb28c8b750d054bc</t>
+  </si>
+  <si>
+    <t>["69c161e5eb28c8b750d054bc"]</t>
+  </si>
+  <si>
+    <t>["Appliances","Visual Displays","Cubicle Curtains"]</t>
+  </si>
+  <si>
+    <t>26-0219</t>
+  </si>
+  <si>
+    <t>Station 33 Bldg 4 Food Hall SD Budget</t>
+  </si>
+  <si>
+    <t>2026-04-17</t>
+  </si>
+  <si>
+    <t>Jonathan Enriquez</t>
+  </si>
+  <si>
+    <t>1256</t>
+  </si>
+  <si>
+    <t>https://app.buildingconnected.com/opportunities/69d403f406964200385d4f8c</t>
+  </si>
+  <si>
+    <t>["69d403f406964200385d4f8c"]</t>
+  </si>
+  <si>
+    <t>["Toilet Accessories","Wall Protection","FEC"]</t>
+  </si>
+  <si>
     <t>26-0218</t>
   </si>
   <si>
@@ -1060,31 +1111,19 @@
     <t>["69d3dce067942824a3512727"]</t>
   </si>
   <si>
-    <t>ATL - Atlanta</t>
-  </si>
-  <si>
-    <t>Declined</t>
-  </si>
-  <si>
-    <t>Joey Dinelli</t>
-  </si>
-  <si>
-    <t>["2026-04-02T22:49:34.183Z: Rejected by Haley Kruse"]</t>
-  </si>
-  <si>
-    <t>26-0195</t>
-  </si>
-  <si>
-    <t>2026-03-26</t>
-  </si>
-  <si>
-    <t>https://app.buildingconnected.com/opportunities/69c161e5eb28c8b750d054bc</t>
-  </si>
-  <si>
-    <t>["69c161e5eb28c8b750d054bc"]</t>
-  </si>
-  <si>
-    <t>["Appliances","Visual Displays","Cubicle Curtains"]</t>
+    <t>26-0217</t>
+  </si>
+  <si>
+    <t>KR</t>
+  </si>
+  <si>
+    <t>https://app.buildingconnected.com/opportunities/69d3de61132a4642c558b4df</t>
+  </si>
+  <si>
+    <t>["69d3de61132a4642c558b4df"]</t>
+  </si>
+  <si>
+    <t>["Lockers"]</t>
   </si>
   <si>
     <t>26-0220</t>
@@ -1111,45 +1150,6 @@
     <t>["69d7cf8f86a4620051a325b4"]</t>
   </si>
   <si>
-    <t>26-0217</t>
-  </si>
-  <si>
-    <t>KR</t>
-  </si>
-  <si>
-    <t>https://app.buildingconnected.com/opportunities/69d3de61132a4642c558b4df</t>
-  </si>
-  <si>
-    <t>["69d3de61132a4642c558b4df"]</t>
-  </si>
-  <si>
-    <t>["Lockers"]</t>
-  </si>
-  <si>
-    <t>26-0219</t>
-  </si>
-  <si>
-    <t>Station 33 Bldg 4 Food Hall SD Budget</t>
-  </si>
-  <si>
-    <t>2026-04-17</t>
-  </si>
-  <si>
-    <t>Jonathan Enriquez</t>
-  </si>
-  <si>
-    <t>1256</t>
-  </si>
-  <si>
-    <t>https://app.buildingconnected.com/opportunities/69d403f406964200385d4f8c</t>
-  </si>
-  <si>
-    <t>["69d403f406964200385d4f8c"]</t>
-  </si>
-  <si>
-    <t>["Toilet Accessories","Wall Protection","FEC"]</t>
-  </si>
-  <si>
     <t>26-0221</t>
   </si>
   <si>
@@ -1327,6 +1327,39 @@
     <t>1146456</t>
   </si>
   <si>
+    <t>26-0198</t>
+  </si>
+  <si>
+    <t>SAN</t>
+  </si>
+  <si>
+    <t>26-0197</t>
+  </si>
+  <si>
+    <t>LAX - FS</t>
+  </si>
+  <si>
+    <t>["Specialties","Storefronts &amp; Curtain Walls"]</t>
+  </si>
+  <si>
+    <t>["Wall Protection","Bike Racks","Cubicle Curtains","Mailbox","Site Furnishing"]</t>
+  </si>
+  <si>
+    <t>["2026-03-31T23:30:11.939Z: scopes added: Storefronts &amp; Curtain Walls"]</t>
+  </si>
+  <si>
+    <t>26-0216</t>
+  </si>
+  <si>
+    <t>https://app.buildingconnected.com/opportunities/69d3e1fe1fa22b68bef01c78</t>
+  </si>
+  <si>
+    <t>["69d3e1fe1fa22b68bef01c78"]</t>
+  </si>
+  <si>
+    <t>["Flagpoles"]</t>
+  </si>
+  <si>
     <t>26-0209</t>
   </si>
   <si>
@@ -1355,39 +1388,6 @@
   </si>
   <si>
     <t>["Sheet Metal &amp; Metal Panels"]</t>
-  </si>
-  <si>
-    <t>26-0198</t>
-  </si>
-  <si>
-    <t>SAN</t>
-  </si>
-  <si>
-    <t>26-0197</t>
-  </si>
-  <si>
-    <t>LAX - FS</t>
-  </si>
-  <si>
-    <t>["Specialties","Storefronts &amp; Curtain Walls"]</t>
-  </si>
-  <si>
-    <t>["Wall Protection","Bike Racks","Cubicle Curtains","Mailbox","Site Furnishing"]</t>
-  </si>
-  <si>
-    <t>["2026-03-31T23:30:11.939Z: scopes added: Storefronts &amp; Curtain Walls"]</t>
-  </si>
-  <si>
-    <t>26-0216</t>
-  </si>
-  <si>
-    <t>https://app.buildingconnected.com/opportunities/69d3e1fe1fa22b68bef01c78</t>
-  </si>
-  <si>
-    <t>["69d3e1fe1fa22b68bef01c78"]</t>
-  </si>
-  <si>
-    <t>["Flagpoles"]</t>
   </si>
   <si>
     <t>26-0028</t>
@@ -5547,49 +5547,49 @@
         <v>123</v>
       </c>
       <c r="C13" t="s">
-        <v>124</v>
+        <v>113</v>
       </c>
       <c r="D13" t="s">
         <v>76</v>
       </c>
       <c r="E13" t="s">
+        <v>124</v>
+      </c>
+      <c r="F13" t="s">
         <v>125</v>
       </c>
-      <c r="F13" t="s">
+      <c r="G13" t="s">
+        <v>45</v>
+      </c>
+      <c r="H13" t="s">
+        <v>45</v>
+      </c>
+      <c r="I13" t="s">
+        <v>45</v>
+      </c>
+      <c r="J13" t="s">
         <v>126</v>
       </c>
-      <c r="G13" t="s">
-        <v>45</v>
-      </c>
-      <c r="H13" t="s">
+      <c r="K13" t="s">
         <v>127</v>
       </c>
-      <c r="I13" t="s">
-        <v>45</v>
-      </c>
-      <c r="J13" t="s">
-        <v>58</v>
-      </c>
-      <c r="K13" t="s">
-        <v>45</v>
-      </c>
       <c r="L13" t="s">
-        <v>45</v>
+        <v>128</v>
       </c>
       <c r="M13" t="s">
         <v>45</v>
       </c>
       <c r="N13" t="s">
-        <v>128</v>
+        <v>45</v>
       </c>
       <c r="O13" t="s">
         <v>45</v>
       </c>
       <c r="P13" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="Q13">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="R13" t="b">
         <v>0</v>
@@ -5604,19 +5604,19 @@
         <v>45</v>
       </c>
       <c r="V13" t="s">
-        <v>129</v>
+        <v>45</v>
       </c>
       <c r="W13" t="s">
-        <v>61</v>
+        <v>45</v>
       </c>
       <c r="X13" t="s">
         <v>45</v>
       </c>
       <c r="Y13" t="s">
-        <v>50</v>
-      </c>
-      <c r="Z13" s="2">
-        <v>46115.811072847224</v>
+        <v>45</v>
+      </c>
+      <c r="Z13" t="s">
+        <v>45</v>
       </c>
       <c r="AA13" t="b">
         <v>0</v>
@@ -5630,73 +5630,73 @@
       <c r="AD13" t="s">
         <v>45</v>
       </c>
-      <c r="AE13" s="2">
-        <v>46121.2517425</v>
+      <c r="AE13" t="s">
+        <v>45</v>
       </c>
       <c r="AF13" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AG13" t="s">
-        <v>41</v>
-      </c>
-      <c r="AH13" s="2">
-        <v>46121.2510297338</v>
+        <v>45</v>
+      </c>
+      <c r="AH13" t="s">
+        <v>45</v>
       </c>
       <c r="AI13" s="2">
-        <v>46115.80864027778</v>
+        <v>46115.64971903936</v>
       </c>
     </row>
     <row r="14" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B14" t="s">
         <v>123</v>
       </c>
       <c r="C14" t="s">
-        <v>113</v>
+        <v>130</v>
       </c>
       <c r="D14" t="s">
         <v>76</v>
       </c>
       <c r="E14" t="s">
+        <v>124</v>
+      </c>
+      <c r="F14" t="s">
         <v>125</v>
       </c>
-      <c r="F14" t="s">
-        <v>126</v>
-      </c>
       <c r="G14" t="s">
         <v>45</v>
       </c>
       <c r="H14" t="s">
-        <v>45</v>
+        <v>131</v>
       </c>
       <c r="I14" t="s">
         <v>45</v>
       </c>
       <c r="J14" t="s">
-        <v>131</v>
+        <v>58</v>
       </c>
       <c r="K14" t="s">
+        <v>45</v>
+      </c>
+      <c r="L14" t="s">
+        <v>45</v>
+      </c>
+      <c r="M14" t="s">
+        <v>45</v>
+      </c>
+      <c r="N14" t="s">
         <v>132</v>
       </c>
-      <c r="L14" t="s">
-        <v>133</v>
-      </c>
-      <c r="M14" t="s">
-        <v>45</v>
-      </c>
-      <c r="N14" t="s">
-        <v>45</v>
-      </c>
       <c r="O14" t="s">
         <v>45</v>
       </c>
       <c r="P14" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="Q14">
-        <v>99</v>
+        <v>107</v>
       </c>
       <c r="R14" t="b">
         <v>0</v>
@@ -5711,19 +5711,19 @@
         <v>45</v>
       </c>
       <c r="V14" t="s">
-        <v>45</v>
+        <v>133</v>
       </c>
       <c r="W14" t="s">
-        <v>45</v>
+        <v>61</v>
       </c>
       <c r="X14" t="s">
         <v>45</v>
       </c>
       <c r="Y14" t="s">
-        <v>45</v>
-      </c>
-      <c r="Z14" t="s">
-        <v>45</v>
+        <v>50</v>
+      </c>
+      <c r="Z14" s="2">
+        <v>46115.811072847224</v>
       </c>
       <c r="AA14" t="b">
         <v>0</v>
@@ -5737,20 +5737,20 @@
       <c r="AD14" t="s">
         <v>45</v>
       </c>
-      <c r="AE14" t="s">
-        <v>45</v>
+      <c r="AE14" s="2">
+        <v>46121.2517425</v>
       </c>
       <c r="AF14" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG14" t="s">
-        <v>45</v>
-      </c>
-      <c r="AH14" t="s">
-        <v>45</v>
+        <v>41</v>
+      </c>
+      <c r="AH14" s="2">
+        <v>46121.2510297338</v>
       </c>
       <c r="AI14" s="2">
-        <v>46115.64971903936</v>
+        <v>46115.80864027778</v>
       </c>
     </row>
     <row r="15" spans="1:35" x14ac:dyDescent="0.25">
@@ -8647,52 +8647,52 @@
         <v>259</v>
       </c>
       <c r="B42" t="s">
-        <v>260</v>
+        <v>172</v>
       </c>
       <c r="C42" t="s">
-        <v>65</v>
+        <v>83</v>
       </c>
       <c r="D42" t="s">
-        <v>200</v>
+        <v>54</v>
       </c>
       <c r="E42" t="s">
+        <v>173</v>
+      </c>
+      <c r="F42" t="s">
+        <v>174</v>
+      </c>
+      <c r="G42" t="s">
+        <v>151</v>
+      </c>
+      <c r="H42" t="s">
+        <v>45</v>
+      </c>
+      <c r="I42" t="s">
+        <v>45</v>
+      </c>
+      <c r="J42" t="s">
+        <v>58</v>
+      </c>
+      <c r="K42" t="s">
         <v>55</v>
       </c>
-      <c r="F42" t="s">
-        <v>210</v>
-      </c>
-      <c r="G42" t="s">
-        <v>45</v>
-      </c>
-      <c r="H42" t="s">
-        <v>261</v>
-      </c>
-      <c r="I42" t="s">
-        <v>262</v>
-      </c>
-      <c r="J42" t="s">
-        <v>44</v>
-      </c>
-      <c r="K42" t="s">
-        <v>45</v>
-      </c>
       <c r="L42" t="s">
-        <v>45</v>
+        <v>175</v>
       </c>
       <c r="M42" t="s">
         <v>45</v>
       </c>
       <c r="N42" t="s">
-        <v>263</v>
+        <v>45</v>
       </c>
       <c r="O42" t="s">
         <v>45</v>
       </c>
       <c r="P42" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="Q42">
-        <v>89</v>
+        <v>77</v>
       </c>
       <c r="R42" t="b">
         <v>0</v>
@@ -8707,19 +8707,19 @@
         <v>45</v>
       </c>
       <c r="V42" t="s">
-        <v>264</v>
+        <v>45</v>
       </c>
       <c r="W42" t="s">
-        <v>61</v>
+        <v>45</v>
       </c>
       <c r="X42" t="s">
-        <v>265</v>
+        <v>45</v>
       </c>
       <c r="Y42" t="s">
-        <v>50</v>
-      </c>
-      <c r="Z42" s="2">
-        <v>46112.95053368056</v>
+        <v>45</v>
+      </c>
+      <c r="Z42" t="s">
+        <v>45</v>
       </c>
       <c r="AA42" t="b">
         <v>0</v>
@@ -8728,13 +8728,13 @@
         <v>45</v>
       </c>
       <c r="AC42" t="s">
-        <v>266</v>
+        <v>45</v>
       </c>
       <c r="AD42" t="s">
         <v>45</v>
       </c>
-      <c r="AE42" t="s">
-        <v>45</v>
+      <c r="AE42" s="2">
+        <v>46093.859216736106</v>
       </c>
       <c r="AF42" t="b">
         <v>0</v>
@@ -8746,60 +8746,60 @@
         <v>45</v>
       </c>
       <c r="AI42" s="2">
-        <v>46112.94978048611</v>
+        <v>46093.82415605324</v>
       </c>
     </row>
     <row r="43" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
+        <v>260</v>
+      </c>
+      <c r="B43" t="s">
+        <v>261</v>
+      </c>
+      <c r="C43" t="s">
+        <v>229</v>
+      </c>
+      <c r="D43" t="s">
+        <v>45</v>
+      </c>
+      <c r="E43" t="s">
+        <v>262</v>
+      </c>
+      <c r="F43" t="s">
+        <v>263</v>
+      </c>
+      <c r="G43" t="s">
+        <v>45</v>
+      </c>
+      <c r="H43" t="s">
+        <v>264</v>
+      </c>
+      <c r="I43" t="s">
+        <v>45</v>
+      </c>
+      <c r="J43" t="s">
+        <v>265</v>
+      </c>
+      <c r="K43" t="s">
+        <v>45</v>
+      </c>
+      <c r="L43" t="s">
+        <v>45</v>
+      </c>
+      <c r="M43" t="s">
+        <v>266</v>
+      </c>
+      <c r="N43" t="s">
         <v>267</v>
       </c>
-      <c r="B43" t="s">
-        <v>172</v>
-      </c>
-      <c r="C43" t="s">
-        <v>83</v>
-      </c>
-      <c r="D43" t="s">
-        <v>54</v>
-      </c>
-      <c r="E43" t="s">
-        <v>173</v>
-      </c>
-      <c r="F43" t="s">
-        <v>174</v>
-      </c>
-      <c r="G43" t="s">
-        <v>151</v>
-      </c>
-      <c r="H43" t="s">
-        <v>45</v>
-      </c>
-      <c r="I43" t="s">
-        <v>45</v>
-      </c>
-      <c r="J43" t="s">
-        <v>58</v>
-      </c>
-      <c r="K43" t="s">
-        <v>55</v>
-      </c>
-      <c r="L43" t="s">
-        <v>175</v>
-      </c>
-      <c r="M43" t="s">
-        <v>45</v>
-      </c>
-      <c r="N43" t="s">
-        <v>45</v>
-      </c>
       <c r="O43" t="s">
         <v>45</v>
       </c>
       <c r="P43" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="Q43">
-        <v>77</v>
+        <v>91</v>
       </c>
       <c r="R43" t="b">
         <v>0</v>
@@ -8814,19 +8814,19 @@
         <v>45</v>
       </c>
       <c r="V43" t="s">
-        <v>45</v>
+        <v>268</v>
       </c>
       <c r="W43" t="s">
-        <v>45</v>
+        <v>269</v>
       </c>
       <c r="X43" t="s">
         <v>45</v>
       </c>
       <c r="Y43" t="s">
-        <v>45</v>
-      </c>
-      <c r="Z43" t="s">
-        <v>45</v>
+        <v>50</v>
+      </c>
+      <c r="Z43" s="2">
+        <v>46112.951310543984</v>
       </c>
       <c r="AA43" t="b">
         <v>0</v>
@@ -8840,8 +8840,8 @@
       <c r="AD43" t="s">
         <v>45</v>
       </c>
-      <c r="AE43" s="2">
-        <v>46093.859216736106</v>
+      <c r="AE43" t="s">
+        <v>45</v>
       </c>
       <c r="AF43" t="b">
         <v>0</v>
@@ -8853,39 +8853,39 @@
         <v>45</v>
       </c>
       <c r="AI43" s="2">
-        <v>46093.82415605324</v>
+        <v>46112.94978027778</v>
       </c>
     </row>
     <row r="44" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="B44" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="C44" t="s">
-        <v>53</v>
+        <v>65</v>
       </c>
       <c r="D44" t="s">
-        <v>45</v>
+        <v>200</v>
       </c>
       <c r="E44" t="s">
-        <v>231</v>
+        <v>55</v>
       </c>
       <c r="F44" t="s">
-        <v>218</v>
+        <v>210</v>
       </c>
       <c r="G44" t="s">
         <v>45</v>
       </c>
       <c r="H44" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="I44" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="J44" t="s">
-        <v>58</v>
+        <v>44</v>
       </c>
       <c r="K44" t="s">
         <v>45</v>
@@ -8897,7 +8897,7 @@
         <v>45</v>
       </c>
       <c r="N44" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="O44" t="s">
         <v>45</v>
@@ -8906,7 +8906,7 @@
         <v>47</v>
       </c>
       <c r="Q44">
-        <v>108</v>
+        <v>89</v>
       </c>
       <c r="R44" t="b">
         <v>0</v>
@@ -8921,28 +8921,28 @@
         <v>45</v>
       </c>
       <c r="V44" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="W44" t="s">
-        <v>274</v>
+        <v>61</v>
       </c>
       <c r="X44" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="Y44" t="s">
         <v>50</v>
       </c>
       <c r="Z44" s="2">
-        <v>46115.811258125</v>
+        <v>46112.95053368056</v>
       </c>
       <c r="AA44" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB44" t="s">
-        <v>276</v>
+        <v>45</v>
       </c>
       <c r="AC44" t="s">
-        <v>45</v>
+        <v>277</v>
       </c>
       <c r="AD44" t="s">
         <v>45</v>
@@ -8960,24 +8960,24 @@
         <v>45</v>
       </c>
       <c r="AI44" s="2">
-        <v>46115.80863989583</v>
+        <v>46112.94978048611</v>
       </c>
     </row>
     <row r="45" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="B45" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="C45" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="D45" t="s">
         <v>54</v>
       </c>
       <c r="E45" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="F45" t="s">
         <v>218</v>
@@ -8986,7 +8986,7 @@
         <v>45</v>
       </c>
       <c r="H45" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="I45" t="s">
         <v>45</v>
@@ -9004,7 +9004,7 @@
         <v>45</v>
       </c>
       <c r="N45" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="O45" t="s">
         <v>45</v>
@@ -9028,13 +9028,13 @@
         <v>45</v>
       </c>
       <c r="V45" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="W45" t="s">
         <v>61</v>
       </c>
       <c r="X45" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="Y45" t="s">
         <v>50</v>
@@ -9072,46 +9072,46 @@
     </row>
     <row r="46" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="B46" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="C46" t="s">
-        <v>229</v>
+        <v>53</v>
       </c>
       <c r="D46" t="s">
         <v>45</v>
       </c>
       <c r="E46" t="s">
-        <v>287</v>
+        <v>231</v>
       </c>
       <c r="F46" t="s">
+        <v>218</v>
+      </c>
+      <c r="G46" t="s">
+        <v>45</v>
+      </c>
+      <c r="H46" t="s">
         <v>288</v>
       </c>
-      <c r="G46" t="s">
-        <v>45</v>
-      </c>
-      <c r="H46" t="s">
+      <c r="I46" t="s">
         <v>289</v>
       </c>
-      <c r="I46" t="s">
-        <v>45</v>
-      </c>
       <c r="J46" t="s">
+        <v>58</v>
+      </c>
+      <c r="K46" t="s">
+        <v>45</v>
+      </c>
+      <c r="L46" t="s">
+        <v>45</v>
+      </c>
+      <c r="M46" t="s">
+        <v>45</v>
+      </c>
+      <c r="N46" t="s">
         <v>290</v>
-      </c>
-      <c r="K46" t="s">
-        <v>45</v>
-      </c>
-      <c r="L46" t="s">
-        <v>45</v>
-      </c>
-      <c r="M46" t="s">
-        <v>291</v>
-      </c>
-      <c r="N46" t="s">
-        <v>292</v>
       </c>
       <c r="O46" t="s">
         <v>45</v>
@@ -9120,7 +9120,7 @@
         <v>47</v>
       </c>
       <c r="Q46">
-        <v>91</v>
+        <v>108</v>
       </c>
       <c r="R46" t="b">
         <v>0</v>
@@ -9135,25 +9135,25 @@
         <v>45</v>
       </c>
       <c r="V46" t="s">
+        <v>291</v>
+      </c>
+      <c r="W46" t="s">
+        <v>292</v>
+      </c>
+      <c r="X46" t="s">
         <v>293</v>
-      </c>
-      <c r="W46" t="s">
-        <v>294</v>
-      </c>
-      <c r="X46" t="s">
-        <v>45</v>
       </c>
       <c r="Y46" t="s">
         <v>50</v>
       </c>
       <c r="Z46" s="2">
-        <v>46112.951310543984</v>
+        <v>46115.811258125</v>
       </c>
       <c r="AA46" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB46" t="s">
-        <v>45</v>
+        <v>294</v>
       </c>
       <c r="AC46" t="s">
         <v>45</v>
@@ -9174,7 +9174,7 @@
         <v>45</v>
       </c>
       <c r="AI46" s="2">
-        <v>46112.94978027778</v>
+        <v>46115.80863989583</v>
       </c>
     </row>
     <row r="47" spans="1:35" x14ac:dyDescent="0.25">
@@ -10463,55 +10463,55 @@
     </row>
     <row r="59" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
+        <v>45</v>
+      </c>
+      <c r="B59" t="s">
+        <v>52</v>
+      </c>
+      <c r="C59" t="s">
         <v>342</v>
       </c>
-      <c r="B59" t="s">
+      <c r="D59" t="s">
+        <v>45</v>
+      </c>
+      <c r="E59" t="s">
+        <v>55</v>
+      </c>
+      <c r="F59" t="s">
+        <v>56</v>
+      </c>
+      <c r="G59" t="s">
+        <v>79</v>
+      </c>
+      <c r="H59" t="s">
+        <v>135</v>
+      </c>
+      <c r="I59" t="s">
+        <v>45</v>
+      </c>
+      <c r="J59" t="s">
         <v>343</v>
       </c>
-      <c r="C59" t="s">
+      <c r="K59" t="s">
+        <v>45</v>
+      </c>
+      <c r="L59" t="s">
+        <v>45</v>
+      </c>
+      <c r="M59" t="s">
+        <v>45</v>
+      </c>
+      <c r="N59" t="s">
+        <v>136</v>
+      </c>
+      <c r="O59" t="s">
         <v>344</v>
-      </c>
-      <c r="D59" t="s">
-        <v>54</v>
-      </c>
-      <c r="E59" t="s">
-        <v>210</v>
-      </c>
-      <c r="F59" t="s">
-        <v>103</v>
-      </c>
-      <c r="G59" t="s">
-        <v>45</v>
-      </c>
-      <c r="H59" t="s">
-        <v>345</v>
-      </c>
-      <c r="I59" t="s">
-        <v>45</v>
-      </c>
-      <c r="J59" t="s">
-        <v>58</v>
-      </c>
-      <c r="K59" t="s">
-        <v>45</v>
-      </c>
-      <c r="L59" t="s">
-        <v>45</v>
-      </c>
-      <c r="M59" t="s">
-        <v>45</v>
-      </c>
-      <c r="N59" t="s">
-        <v>346</v>
-      </c>
-      <c r="O59" t="s">
-        <v>45</v>
       </c>
       <c r="P59" t="s">
         <v>47</v>
       </c>
-      <c r="Q59">
-        <v>112</v>
+      <c r="Q59" t="s">
+        <v>45</v>
       </c>
       <c r="R59" t="b">
         <v>0</v>
@@ -10526,25 +10526,25 @@
         <v>45</v>
       </c>
       <c r="V59" t="s">
-        <v>347</v>
+        <v>137</v>
       </c>
       <c r="W59" t="s">
-        <v>61</v>
+        <v>138</v>
       </c>
       <c r="X59" t="s">
         <v>45</v>
       </c>
       <c r="Y59" t="s">
-        <v>50</v>
-      </c>
-      <c r="Z59" s="2">
-        <v>46120.75758967592</v>
+        <v>45</v>
+      </c>
+      <c r="Z59" t="s">
+        <v>45</v>
       </c>
       <c r="AA59" t="b">
         <v>0</v>
       </c>
       <c r="AB59" t="s">
-        <v>45</v>
+        <v>345</v>
       </c>
       <c r="AC59" t="s">
         <v>45</v>
@@ -10552,8 +10552,8 @@
       <c r="AD59" t="s">
         <v>45</v>
       </c>
-      <c r="AE59" t="s">
-        <v>45</v>
+      <c r="AE59" s="2">
+        <v>46114.95109008102</v>
       </c>
       <c r="AF59" t="b">
         <v>0</v>
@@ -10565,60 +10565,60 @@
         <v>45</v>
       </c>
       <c r="AI59" s="2">
-        <v>46120.75685143519</v>
+        <v>46113.82840027778</v>
       </c>
     </row>
     <row r="60" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>45</v>
+        <v>346</v>
       </c>
       <c r="B60" t="s">
-        <v>52</v>
+        <v>287</v>
       </c>
       <c r="C60" t="s">
+        <v>45</v>
+      </c>
+      <c r="D60" t="s">
+        <v>54</v>
+      </c>
+      <c r="E60" t="s">
+        <v>347</v>
+      </c>
+      <c r="F60" t="s">
+        <v>263</v>
+      </c>
+      <c r="G60" t="s">
+        <v>45</v>
+      </c>
+      <c r="H60" t="s">
+        <v>288</v>
+      </c>
+      <c r="I60" t="s">
+        <v>45</v>
+      </c>
+      <c r="J60" t="s">
+        <v>58</v>
+      </c>
+      <c r="K60" t="s">
+        <v>45</v>
+      </c>
+      <c r="L60" t="s">
+        <v>45</v>
+      </c>
+      <c r="M60" t="s">
+        <v>45</v>
+      </c>
+      <c r="N60" t="s">
         <v>348</v>
       </c>
-      <c r="D60" t="s">
-        <v>45</v>
-      </c>
-      <c r="E60" t="s">
-        <v>55</v>
-      </c>
-      <c r="F60" t="s">
-        <v>56</v>
-      </c>
-      <c r="G60" t="s">
-        <v>79</v>
-      </c>
-      <c r="H60" t="s">
-        <v>135</v>
-      </c>
-      <c r="I60" t="s">
-        <v>45</v>
-      </c>
-      <c r="J60" t="s">
-        <v>349</v>
-      </c>
-      <c r="K60" t="s">
-        <v>45</v>
-      </c>
-      <c r="L60" t="s">
-        <v>45</v>
-      </c>
-      <c r="M60" t="s">
-        <v>45</v>
-      </c>
-      <c r="N60" t="s">
-        <v>136</v>
-      </c>
       <c r="O60" t="s">
-        <v>350</v>
+        <v>45</v>
       </c>
       <c r="P60" t="s">
         <v>47</v>
       </c>
-      <c r="Q60" t="s">
-        <v>45</v>
+      <c r="Q60">
+        <v>90</v>
       </c>
       <c r="R60" t="b">
         <v>0</v>
@@ -10633,25 +10633,25 @@
         <v>45</v>
       </c>
       <c r="V60" t="s">
-        <v>137</v>
+        <v>349</v>
       </c>
       <c r="W60" t="s">
-        <v>138</v>
+        <v>61</v>
       </c>
       <c r="X60" t="s">
-        <v>45</v>
+        <v>350</v>
       </c>
       <c r="Y60" t="s">
-        <v>45</v>
-      </c>
-      <c r="Z60" t="s">
-        <v>45</v>
+        <v>50</v>
+      </c>
+      <c r="Z60" s="2">
+        <v>46112.951018148146</v>
       </c>
       <c r="AA60" t="b">
         <v>0</v>
       </c>
       <c r="AB60" t="s">
-        <v>351</v>
+        <v>45</v>
       </c>
       <c r="AC60" t="s">
         <v>45</v>
@@ -10660,7 +10660,7 @@
         <v>45</v>
       </c>
       <c r="AE60" s="2">
-        <v>46114.95109008102</v>
+        <v>46113.94965768518</v>
       </c>
       <c r="AF60" t="b">
         <v>0</v>
@@ -10672,36 +10672,36 @@
         <v>45</v>
       </c>
       <c r="AI60" s="2">
-        <v>46113.82840027778</v>
+        <v>46112.94978038194</v>
       </c>
     </row>
     <row r="61" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
+        <v>351</v>
+      </c>
+      <c r="B61" t="s">
         <v>352</v>
       </c>
-      <c r="B61" t="s">
-        <v>269</v>
-      </c>
       <c r="C61" t="s">
-        <v>45</v>
+        <v>130</v>
       </c>
       <c r="D61" t="s">
         <v>54</v>
       </c>
       <c r="E61" t="s">
+        <v>263</v>
+      </c>
+      <c r="F61" t="s">
         <v>353</v>
       </c>
-      <c r="F61" t="s">
-        <v>288</v>
-      </c>
       <c r="G61" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="H61" t="s">
-        <v>270</v>
+        <v>354</v>
       </c>
       <c r="I61" t="s">
-        <v>45</v>
+        <v>355</v>
       </c>
       <c r="J61" t="s">
         <v>58</v>
@@ -10716,7 +10716,7 @@
         <v>45</v>
       </c>
       <c r="N61" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="O61" t="s">
         <v>45</v>
@@ -10725,7 +10725,7 @@
         <v>47</v>
       </c>
       <c r="Q61">
-        <v>90</v>
+        <v>113</v>
       </c>
       <c r="R61" t="b">
         <v>0</v>
@@ -10740,19 +10740,19 @@
         <v>45</v>
       </c>
       <c r="V61" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="W61" t="s">
         <v>61</v>
       </c>
       <c r="X61" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="Y61" t="s">
         <v>50</v>
       </c>
       <c r="Z61" s="2">
-        <v>46112.951018148146</v>
+        <v>46120.75803053241</v>
       </c>
       <c r="AA61" t="b">
         <v>0</v>
@@ -10766,8 +10766,8 @@
       <c r="AD61" t="s">
         <v>45</v>
       </c>
-      <c r="AE61" s="2">
-        <v>46113.94965768518</v>
+      <c r="AE61" t="s">
+        <v>45</v>
       </c>
       <c r="AF61" t="b">
         <v>0</v>
@@ -10779,39 +10779,39 @@
         <v>45</v>
       </c>
       <c r="AI61" s="2">
-        <v>46112.94978038194</v>
+        <v>46120.756850844904</v>
       </c>
     </row>
     <row r="62" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="B62" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="C62" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="D62" t="s">
         <v>54</v>
       </c>
       <c r="E62" t="s">
-        <v>56</v>
+        <v>210</v>
       </c>
       <c r="F62" t="s">
-        <v>360</v>
+        <v>103</v>
       </c>
       <c r="G62" t="s">
         <v>45</v>
       </c>
       <c r="H62" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="I62" t="s">
         <v>45</v>
       </c>
       <c r="J62" t="s">
-        <v>362</v>
+        <v>58</v>
       </c>
       <c r="K62" t="s">
         <v>45</v>
@@ -10831,8 +10831,8 @@
       <c r="P62" t="s">
         <v>47</v>
       </c>
-      <c r="Q62" t="s">
-        <v>45</v>
+      <c r="Q62">
+        <v>112</v>
       </c>
       <c r="R62" t="b">
         <v>0</v>
@@ -10841,7 +10841,7 @@
         <v>1</v>
       </c>
       <c r="T62" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U62" t="s">
         <v>45</v>
@@ -10856,10 +10856,10 @@
         <v>45</v>
       </c>
       <c r="Y62" t="s">
-        <v>45</v>
-      </c>
-      <c r="Z62" t="s">
-        <v>45</v>
+        <v>50</v>
+      </c>
+      <c r="Z62" s="2">
+        <v>46120.75758967592</v>
       </c>
       <c r="AA62" t="b">
         <v>0</v>
@@ -10886,7 +10886,7 @@
         <v>45</v>
       </c>
       <c r="AI62" s="2">
-        <v>46121.80852202546</v>
+        <v>46120.75685143519</v>
       </c>
     </row>
     <row r="63" spans="1:35" x14ac:dyDescent="0.25">
@@ -10894,10 +10894,10 @@
         <v>365</v>
       </c>
       <c r="B63" t="s">
-        <v>343</v>
+        <v>360</v>
       </c>
       <c r="C63" t="s">
-        <v>344</v>
+        <v>361</v>
       </c>
       <c r="D63" t="s">
         <v>54</v>
@@ -10912,7 +10912,7 @@
         <v>366</v>
       </c>
       <c r="H63" t="s">
-        <v>345</v>
+        <v>362</v>
       </c>
       <c r="I63" t="s">
         <v>45</v>
@@ -11004,28 +11004,28 @@
         <v>371</v>
       </c>
       <c r="C64" t="s">
-        <v>124</v>
+        <v>372</v>
       </c>
       <c r="D64" t="s">
         <v>54</v>
       </c>
       <c r="E64" t="s">
-        <v>288</v>
+        <v>56</v>
       </c>
       <c r="F64" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="G64" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="H64" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="I64" t="s">
-        <v>374</v>
+        <v>45</v>
       </c>
       <c r="J64" t="s">
-        <v>58</v>
+        <v>375</v>
       </c>
       <c r="K64" t="s">
         <v>45</v>
@@ -11037,7 +11037,7 @@
         <v>45</v>
       </c>
       <c r="N64" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="O64" t="s">
         <v>45</v>
@@ -11045,8 +11045,8 @@
       <c r="P64" t="s">
         <v>47</v>
       </c>
-      <c r="Q64">
-        <v>113</v>
+      <c r="Q64" t="s">
+        <v>45</v>
       </c>
       <c r="R64" t="b">
         <v>0</v>
@@ -11055,25 +11055,25 @@
         <v>1</v>
       </c>
       <c r="T64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U64" t="s">
         <v>45</v>
       </c>
       <c r="V64" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="W64" t="s">
         <v>61</v>
       </c>
       <c r="X64" t="s">
-        <v>377</v>
+        <v>45</v>
       </c>
       <c r="Y64" t="s">
-        <v>50</v>
-      </c>
-      <c r="Z64" s="2">
-        <v>46120.75803053241</v>
+        <v>45</v>
+      </c>
+      <c r="Z64" t="s">
+        <v>45</v>
       </c>
       <c r="AA64" t="b">
         <v>0</v>
@@ -11100,7 +11100,7 @@
         <v>45</v>
       </c>
       <c r="AI64" s="2">
-        <v>46120.756850844904</v>
+        <v>46121.80852202546</v>
       </c>
     </row>
     <row r="65" spans="1:35" x14ac:dyDescent="0.25">
@@ -11120,7 +11120,7 @@
         <v>56</v>
       </c>
       <c r="F65" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G65" t="s">
         <v>45</v>
@@ -11132,7 +11132,7 @@
         <v>45</v>
       </c>
       <c r="J65" t="s">
-        <v>362</v>
+        <v>375</v>
       </c>
       <c r="K65" t="s">
         <v>45</v>
@@ -11539,7 +11539,7 @@
         <v>397</v>
       </c>
       <c r="C69" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="D69" t="s">
         <v>54</v>
@@ -11548,7 +11548,7 @@
         <v>185</v>
       </c>
       <c r="F69" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="G69" t="s">
         <v>45</v>
@@ -11646,7 +11646,7 @@
         <v>399</v>
       </c>
       <c r="C70" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="D70" t="s">
         <v>114</v>
@@ -12074,7 +12074,7 @@
         <v>415</v>
       </c>
       <c r="C74" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="D74" t="s">
         <v>54</v>
@@ -12606,7 +12606,7 @@
         <v>437</v>
       </c>
       <c r="B79" t="s">
-        <v>278</v>
+        <v>100</v>
       </c>
       <c r="C79" t="s">
         <v>438</v>
@@ -12615,16 +12615,16 @@
         <v>54</v>
       </c>
       <c r="E79" t="s">
-        <v>280</v>
+        <v>102</v>
       </c>
       <c r="F79" t="s">
-        <v>218</v>
+        <v>103</v>
       </c>
       <c r="G79" t="s">
-        <v>366</v>
+        <v>45</v>
       </c>
       <c r="H79" t="s">
-        <v>281</v>
+        <v>104</v>
       </c>
       <c r="I79" t="s">
         <v>45</v>
@@ -12642,7 +12642,7 @@
         <v>45</v>
       </c>
       <c r="N79" t="s">
-        <v>282</v>
+        <v>107</v>
       </c>
       <c r="O79" t="s">
         <v>45</v>
@@ -12651,7 +12651,7 @@
         <v>47</v>
       </c>
       <c r="Q79">
-        <v>103</v>
+        <v>93</v>
       </c>
       <c r="R79" t="b">
         <v>0</v>
@@ -12666,7 +12666,7 @@
         <v>45</v>
       </c>
       <c r="V79" t="s">
-        <v>283</v>
+        <v>108</v>
       </c>
       <c r="W79" t="s">
         <v>61</v>
@@ -12678,7 +12678,7 @@
         <v>50</v>
       </c>
       <c r="Z79" s="2">
-        <v>46115.81067839121</v>
+        <v>46112.95175853009</v>
       </c>
       <c r="AA79" t="b">
         <v>0</v>
@@ -12692,8 +12692,8 @@
       <c r="AD79" t="s">
         <v>45</v>
       </c>
-      <c r="AE79" t="s">
-        <v>45</v>
+      <c r="AE79" s="2">
+        <v>46113.94965768518</v>
       </c>
       <c r="AF79" t="b">
         <v>0</v>
@@ -12705,7 +12705,7 @@
         <v>45</v>
       </c>
       <c r="AI79" s="2">
-        <v>46115.808641111114</v>
+        <v>46112.94978008102</v>
       </c>
     </row>
     <row r="80" spans="1:35" x14ac:dyDescent="0.25">
@@ -12713,28 +12713,28 @@
         <v>439</v>
       </c>
       <c r="B80" t="s">
+        <v>36</v>
+      </c>
+      <c r="C80" t="s">
         <v>440</v>
       </c>
-      <c r="C80" t="s">
-        <v>37</v>
-      </c>
       <c r="D80" t="s">
-        <v>441</v>
+        <v>38</v>
       </c>
       <c r="E80" t="s">
-        <v>102</v>
+        <v>39</v>
       </c>
       <c r="F80" t="s">
-        <v>287</v>
+        <v>40</v>
       </c>
       <c r="G80" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="H80" t="s">
-        <v>442</v>
+        <v>42</v>
       </c>
       <c r="I80" t="s">
-        <v>443</v>
+        <v>45</v>
       </c>
       <c r="J80" t="s">
         <v>58</v>
@@ -12749,7 +12749,7 @@
         <v>45</v>
       </c>
       <c r="N80" t="s">
-        <v>444</v>
+        <v>46</v>
       </c>
       <c r="O80" t="s">
         <v>45</v>
@@ -12758,7 +12758,7 @@
         <v>47</v>
       </c>
       <c r="Q80">
-        <v>102</v>
+        <v>92</v>
       </c>
       <c r="R80" t="b">
         <v>0</v>
@@ -12773,25 +12773,25 @@
         <v>45</v>
       </c>
       <c r="V80" t="s">
-        <v>445</v>
+        <v>48</v>
       </c>
       <c r="W80" t="s">
-        <v>446</v>
+        <v>441</v>
       </c>
       <c r="X80" t="s">
-        <v>109</v>
+        <v>442</v>
       </c>
       <c r="Y80" t="s">
         <v>50</v>
       </c>
       <c r="Z80" s="2">
-        <v>46115.810453784725</v>
+        <v>46112.951662962965</v>
       </c>
       <c r="AA80" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB80" t="s">
-        <v>45</v>
+        <v>443</v>
       </c>
       <c r="AC80" t="s">
         <v>45</v>
@@ -12799,8 +12799,8 @@
       <c r="AD80" t="s">
         <v>45</v>
       </c>
-      <c r="AE80" t="s">
-        <v>45</v>
+      <c r="AE80" s="2">
+        <v>46113.94965768518</v>
       </c>
       <c r="AF80" t="b">
         <v>0</v>
@@ -12812,24 +12812,24 @@
         <v>45</v>
       </c>
       <c r="AI80" s="2">
-        <v>46115.80864127315</v>
+        <v>46112.949780173614</v>
       </c>
     </row>
     <row r="81" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>447</v>
+        <v>444</v>
       </c>
       <c r="B81" t="s">
-        <v>100</v>
+        <v>360</v>
       </c>
       <c r="C81" t="s">
-        <v>448</v>
+        <v>361</v>
       </c>
       <c r="D81" t="s">
         <v>54</v>
       </c>
       <c r="E81" t="s">
-        <v>102</v>
+        <v>210</v>
       </c>
       <c r="F81" t="s">
         <v>103</v>
@@ -12838,10 +12838,10 @@
         <v>45</v>
       </c>
       <c r="H81" t="s">
-        <v>104</v>
+        <v>362</v>
       </c>
       <c r="I81" t="s">
-        <v>45</v>
+        <v>289</v>
       </c>
       <c r="J81" t="s">
         <v>58</v>
@@ -12856,7 +12856,7 @@
         <v>45</v>
       </c>
       <c r="N81" t="s">
-        <v>107</v>
+        <v>445</v>
       </c>
       <c r="O81" t="s">
         <v>45</v>
@@ -12865,7 +12865,7 @@
         <v>47</v>
       </c>
       <c r="Q81">
-        <v>93</v>
+        <v>110</v>
       </c>
       <c r="R81" t="b">
         <v>0</v>
@@ -12880,10 +12880,10 @@
         <v>45</v>
       </c>
       <c r="V81" t="s">
-        <v>108</v>
+        <v>446</v>
       </c>
       <c r="W81" t="s">
-        <v>61</v>
+        <v>447</v>
       </c>
       <c r="X81" t="s">
         <v>45</v>
@@ -12892,7 +12892,7 @@
         <v>50</v>
       </c>
       <c r="Z81" s="2">
-        <v>46112.95175853009</v>
+        <v>46118.958962268516</v>
       </c>
       <c r="AA81" t="b">
         <v>0</v>
@@ -12907,45 +12907,45 @@
         <v>45</v>
       </c>
       <c r="AE81" s="2">
-        <v>46113.94965768518</v>
+        <v>46121.252319861116</v>
       </c>
       <c r="AF81" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG81" t="s">
-        <v>45</v>
-      </c>
-      <c r="AH81" t="s">
-        <v>45</v>
+        <v>79</v>
+      </c>
+      <c r="AH81" s="2">
+        <v>46121.25048729166</v>
       </c>
       <c r="AI81" s="2">
-        <v>46112.94978008102</v>
+        <v>46118.957825254634</v>
       </c>
     </row>
     <row r="82" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
+        <v>448</v>
+      </c>
+      <c r="B82" t="s">
+        <v>279</v>
+      </c>
+      <c r="C82" t="s">
         <v>449</v>
       </c>
-      <c r="B82" t="s">
-        <v>36</v>
-      </c>
-      <c r="C82" t="s">
-        <v>450</v>
-      </c>
       <c r="D82" t="s">
-        <v>38</v>
+        <v>54</v>
       </c>
       <c r="E82" t="s">
-        <v>39</v>
+        <v>281</v>
       </c>
       <c r="F82" t="s">
-        <v>40</v>
+        <v>218</v>
       </c>
       <c r="G82" t="s">
-        <v>45</v>
+        <v>366</v>
       </c>
       <c r="H82" t="s">
-        <v>42</v>
+        <v>282</v>
       </c>
       <c r="I82" t="s">
         <v>45</v>
@@ -12963,7 +12963,7 @@
         <v>45</v>
       </c>
       <c r="N82" t="s">
-        <v>46</v>
+        <v>283</v>
       </c>
       <c r="O82" t="s">
         <v>45</v>
@@ -12972,7 +12972,7 @@
         <v>47</v>
       </c>
       <c r="Q82">
-        <v>92</v>
+        <v>103</v>
       </c>
       <c r="R82" t="b">
         <v>0</v>
@@ -12987,25 +12987,25 @@
         <v>45</v>
       </c>
       <c r="V82" t="s">
-        <v>48</v>
+        <v>284</v>
       </c>
       <c r="W82" t="s">
-        <v>451</v>
+        <v>61</v>
       </c>
       <c r="X82" t="s">
-        <v>452</v>
+        <v>45</v>
       </c>
       <c r="Y82" t="s">
         <v>50</v>
       </c>
       <c r="Z82" s="2">
-        <v>46112.951662962965</v>
+        <v>46115.81067839121</v>
       </c>
       <c r="AA82" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB82" t="s">
-        <v>453</v>
+        <v>45</v>
       </c>
       <c r="AC82" t="s">
         <v>45</v>
@@ -13013,8 +13013,8 @@
       <c r="AD82" t="s">
         <v>45</v>
       </c>
-      <c r="AE82" s="2">
-        <v>46113.94965768518</v>
+      <c r="AE82" t="s">
+        <v>45</v>
       </c>
       <c r="AF82" t="b">
         <v>0</v>
@@ -13026,36 +13026,36 @@
         <v>45</v>
       </c>
       <c r="AI82" s="2">
-        <v>46112.949780173614</v>
+        <v>46115.808641111114</v>
       </c>
     </row>
     <row r="83" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
+        <v>450</v>
+      </c>
+      <c r="B83" t="s">
+        <v>451</v>
+      </c>
+      <c r="C83" t="s">
+        <v>37</v>
+      </c>
+      <c r="D83" t="s">
+        <v>452</v>
+      </c>
+      <c r="E83" t="s">
+        <v>102</v>
+      </c>
+      <c r="F83" t="s">
+        <v>262</v>
+      </c>
+      <c r="G83" t="s">
+        <v>41</v>
+      </c>
+      <c r="H83" t="s">
+        <v>453</v>
+      </c>
+      <c r="I83" t="s">
         <v>454</v>
-      </c>
-      <c r="B83" t="s">
-        <v>343</v>
-      </c>
-      <c r="C83" t="s">
-        <v>344</v>
-      </c>
-      <c r="D83" t="s">
-        <v>54</v>
-      </c>
-      <c r="E83" t="s">
-        <v>210</v>
-      </c>
-      <c r="F83" t="s">
-        <v>103</v>
-      </c>
-      <c r="G83" t="s">
-        <v>45</v>
-      </c>
-      <c r="H83" t="s">
-        <v>345</v>
-      </c>
-      <c r="I83" t="s">
-        <v>271</v>
       </c>
       <c r="J83" t="s">
         <v>58</v>
@@ -13079,7 +13079,7 @@
         <v>47</v>
       </c>
       <c r="Q83">
-        <v>110</v>
+        <v>102</v>
       </c>
       <c r="R83" t="b">
         <v>0</v>
@@ -13100,13 +13100,13 @@
         <v>457</v>
       </c>
       <c r="X83" t="s">
-        <v>45</v>
+        <v>109</v>
       </c>
       <c r="Y83" t="s">
         <v>50</v>
       </c>
       <c r="Z83" s="2">
-        <v>46118.958962268516</v>
+        <v>46115.810453784725</v>
       </c>
       <c r="AA83" t="b">
         <v>0</v>
@@ -13120,20 +13120,20 @@
       <c r="AD83" t="s">
         <v>45</v>
       </c>
-      <c r="AE83" s="2">
-        <v>46121.252319861116</v>
+      <c r="AE83" t="s">
+        <v>45</v>
       </c>
       <c r="AF83" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AG83" t="s">
-        <v>79</v>
-      </c>
-      <c r="AH83" s="2">
-        <v>46121.25048729166</v>
+        <v>45</v>
+      </c>
+      <c r="AH83" t="s">
+        <v>45</v>
       </c>
       <c r="AI83" s="2">
-        <v>46118.957825254634</v>
+        <v>46115.80864127315</v>
       </c>
     </row>
     <row r="84" spans="1:35" x14ac:dyDescent="0.25">
@@ -13896,7 +13896,7 @@
         <v>217</v>
       </c>
       <c r="D91" t="s">
-        <v>441</v>
+        <v>452</v>
       </c>
       <c r="E91" t="s">
         <v>155</v>
@@ -14211,7 +14211,7 @@
         <v>502</v>
       </c>
       <c r="B94" t="s">
-        <v>440</v>
+        <v>451</v>
       </c>
       <c r="C94" t="s">
         <v>37</v>
@@ -14223,13 +14223,13 @@
         <v>102</v>
       </c>
       <c r="F94" t="s">
-        <v>287</v>
+        <v>262</v>
       </c>
       <c r="G94" t="s">
         <v>45</v>
       </c>
       <c r="H94" t="s">
-        <v>442</v>
+        <v>453</v>
       </c>
       <c r="I94" t="s">
         <v>45</v>
@@ -14247,7 +14247,7 @@
         <v>504</v>
       </c>
       <c r="N94" t="s">
-        <v>444</v>
+        <v>455</v>
       </c>
       <c r="O94" t="s">
         <v>45</v>
@@ -14271,10 +14271,10 @@
         <v>45</v>
       </c>
       <c r="V94" t="s">
-        <v>445</v>
+        <v>456</v>
       </c>
       <c r="W94" t="s">
-        <v>446</v>
+        <v>457</v>
       </c>
       <c r="X94" t="s">
         <v>505</v>
@@ -14749,10 +14749,10 @@
         <v>524</v>
       </c>
       <c r="C99" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="D99" t="s">
-        <v>441</v>
+        <v>452</v>
       </c>
       <c r="E99" t="s">
         <v>174</v>
@@ -15406,7 +15406,7 @@
         <v>79</v>
       </c>
       <c r="H105" t="s">
-        <v>361</v>
+        <v>374</v>
       </c>
       <c r="I105" t="s">
         <v>546</v>
@@ -15620,7 +15620,7 @@
         <v>41</v>
       </c>
       <c r="H107" t="s">
-        <v>361</v>
+        <v>374</v>
       </c>
       <c r="I107" t="s">
         <v>554</v>
@@ -15718,22 +15718,22 @@
         <v>76</v>
       </c>
       <c r="E108" t="s">
+        <v>124</v>
+      </c>
+      <c r="F108" t="s">
         <v>125</v>
       </c>
-      <c r="F108" t="s">
-        <v>126</v>
-      </c>
       <c r="G108" t="s">
         <v>45</v>
       </c>
       <c r="H108" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="I108" t="s">
         <v>45</v>
       </c>
       <c r="J108" t="s">
-        <v>349</v>
+        <v>343</v>
       </c>
       <c r="K108" t="s">
         <v>45</v>
@@ -15745,7 +15745,7 @@
         <v>45</v>
       </c>
       <c r="N108" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="O108" t="s">
         <v>45</v>
@@ -15769,7 +15769,7 @@
         <v>45</v>
       </c>
       <c r="V108" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="W108" t="s">
         <v>61</v>
@@ -15929,7 +15929,7 @@
         <v>299</v>
       </c>
       <c r="D110" t="s">
-        <v>441</v>
+        <v>452</v>
       </c>
       <c r="E110" t="s">
         <v>155</v>
@@ -16149,7 +16149,7 @@
         <v>155</v>
       </c>
       <c r="F112" t="s">
-        <v>287</v>
+        <v>262</v>
       </c>
       <c r="G112" t="s">
         <v>41</v>
@@ -16470,7 +16470,7 @@
         <v>194</v>
       </c>
       <c r="F115" t="s">
-        <v>287</v>
+        <v>262</v>
       </c>
       <c r="G115" t="s">
         <v>79</v>
@@ -16678,7 +16678,7 @@
         <v>149</v>
       </c>
       <c r="D117" t="s">
-        <v>441</v>
+        <v>452</v>
       </c>
       <c r="E117" t="s">
         <v>155</v>
@@ -16889,7 +16889,7 @@
         <v>587</v>
       </c>
       <c r="C119" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="D119" t="s">
         <v>142</v>
@@ -17852,7 +17852,7 @@
         <v>399</v>
       </c>
       <c r="C128" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="D128" t="s">
         <v>114</v>
@@ -18509,7 +18509,7 @@
         <v>151</v>
       </c>
       <c r="H134" t="s">
-        <v>361</v>
+        <v>374</v>
       </c>
       <c r="I134" t="s">
         <v>643</v>
@@ -20741,7 +20741,7 @@
         <v>704</v>
       </c>
       <c r="C155" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="D155" t="s">
         <v>54</v>
@@ -22563,7 +22563,7 @@
         <v>221</v>
       </c>
       <c r="D172" t="s">
-        <v>441</v>
+        <v>452</v>
       </c>
       <c r="E172" t="s">
         <v>155</v>
@@ -23630,7 +23630,7 @@
         <v>785</v>
       </c>
       <c r="C182" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="D182" t="s">
         <v>54</v>
@@ -23639,7 +23639,7 @@
         <v>194</v>
       </c>
       <c r="F182" t="s">
-        <v>353</v>
+        <v>347</v>
       </c>
       <c r="G182" t="s">
         <v>79</v>
@@ -23844,7 +23844,7 @@
         <v>792</v>
       </c>
       <c r="C184" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="D184" t="s">
         <v>54</v>
@@ -25571,7 +25571,7 @@
         <v>151</v>
       </c>
       <c r="H200" t="s">
-        <v>361</v>
+        <v>374</v>
       </c>
       <c r="I200" t="s">
         <v>850</v>
@@ -25770,7 +25770,7 @@
         <v>856</v>
       </c>
       <c r="C202" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="D202" t="s">
         <v>142</v>
@@ -26213,7 +26213,7 @@
         <v>151</v>
       </c>
       <c r="H206" t="s">
-        <v>361</v>
+        <v>374</v>
       </c>
       <c r="I206" t="s">
         <v>871</v>
@@ -27378,7 +27378,7 @@
         <v>149</v>
       </c>
       <c r="D217" t="s">
-        <v>441</v>
+        <v>452</v>
       </c>
       <c r="E217" t="s">
         <v>155</v>
@@ -27598,7 +27598,7 @@
         <v>155</v>
       </c>
       <c r="F219" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="G219" t="s">
         <v>41</v>
@@ -27699,7 +27699,7 @@
         <v>303</v>
       </c>
       <c r="D220" t="s">
-        <v>441</v>
+        <v>452</v>
       </c>
       <c r="E220" t="s">
         <v>155</v>
@@ -28133,7 +28133,7 @@
         <v>155</v>
       </c>
       <c r="F224" t="s">
-        <v>287</v>
+        <v>262</v>
       </c>
       <c r="G224" t="s">
         <v>79</v>
@@ -28231,7 +28231,7 @@
         <v>415</v>
       </c>
       <c r="C225" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="D225" t="s">
         <v>54</v>
@@ -28775,7 +28775,7 @@
         <v>155</v>
       </c>
       <c r="F230" t="s">
-        <v>287</v>
+        <v>262</v>
       </c>
       <c r="G230" t="s">
         <v>79</v>
@@ -31016,7 +31016,7 @@
         <v>149</v>
       </c>
       <c r="D251" t="s">
-        <v>441</v>
+        <v>452</v>
       </c>
       <c r="E251" t="s">
         <v>155</v>
@@ -32086,7 +32086,7 @@
         <v>299</v>
       </c>
       <c r="D261" t="s">
-        <v>441</v>
+        <v>452</v>
       </c>
       <c r="E261" t="s">
         <v>155</v>
@@ -32407,7 +32407,7 @@
         <v>217</v>
       </c>
       <c r="D264" t="s">
-        <v>441</v>
+        <v>452</v>
       </c>
       <c r="E264" t="s">
         <v>155</v>
@@ -32511,7 +32511,7 @@
         <v>792</v>
       </c>
       <c r="C265" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="D265" t="s">
         <v>54</v>
@@ -33263,7 +33263,7 @@
         <v>149</v>
       </c>
       <c r="D272" t="s">
-        <v>441</v>
+        <v>452</v>
       </c>
       <c r="E272" t="s">
         <v>155</v>
@@ -34238,7 +34238,7 @@
         <v>151</v>
       </c>
       <c r="H281" t="s">
-        <v>361</v>
+        <v>374</v>
       </c>
       <c r="I281" t="s">
         <v>643</v>
@@ -34330,7 +34330,7 @@
         <v>704</v>
       </c>
       <c r="C282" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="D282" t="s">
         <v>54</v>
@@ -34773,10 +34773,10 @@
         <v>79</v>
       </c>
       <c r="H286" t="s">
-        <v>361</v>
+        <v>374</v>
       </c>
       <c r="I286" t="s">
-        <v>271</v>
+        <v>289</v>
       </c>
       <c r="J286" t="s">
         <v>58</v>
@@ -34865,7 +34865,7 @@
         <v>587</v>
       </c>
       <c r="C287" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="D287" t="s">
         <v>142</v>
@@ -34972,7 +34972,7 @@
         <v>856</v>
       </c>
       <c r="C288" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="D288" t="s">
         <v>142</v>
@@ -36806,7 +36806,7 @@
         <v>151</v>
       </c>
       <c r="H305" t="s">
-        <v>361</v>
+        <v>374</v>
       </c>
       <c r="I305" t="s">
         <v>850</v>
@@ -36913,7 +36913,7 @@
         <v>41</v>
       </c>
       <c r="H306" t="s">
-        <v>361</v>
+        <v>374</v>
       </c>
       <c r="I306" t="s">
         <v>554</v>
@@ -37442,7 +37442,7 @@
         <v>155</v>
       </c>
       <c r="F311" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="G311" t="s">
         <v>41</v>
@@ -37977,7 +37977,7 @@
         <v>155</v>
       </c>
       <c r="F316" t="s">
-        <v>287</v>
+        <v>262</v>
       </c>
       <c r="G316" t="s">
         <v>79</v>
@@ -38506,7 +38506,7 @@
         <v>303</v>
       </c>
       <c r="D321" t="s">
-        <v>441</v>
+        <v>452</v>
       </c>
       <c r="E321" t="s">
         <v>155</v>
@@ -39261,7 +39261,7 @@
         <v>155</v>
       </c>
       <c r="F328" t="s">
-        <v>287</v>
+        <v>262</v>
       </c>
       <c r="G328" t="s">
         <v>41</v>
@@ -39787,7 +39787,7 @@
         <v>1055</v>
       </c>
       <c r="C333" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="D333" t="s">
         <v>200</v>
@@ -40117,7 +40117,7 @@
         <v>155</v>
       </c>
       <c r="F336" t="s">
-        <v>287</v>
+        <v>262</v>
       </c>
       <c r="G336" t="s">
         <v>79</v>
@@ -40643,7 +40643,7 @@
         <v>1066</v>
       </c>
       <c r="C341" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="D341" t="s">
         <v>54</v>
@@ -41074,7 +41074,7 @@
         <v>221</v>
       </c>
       <c r="D345" t="s">
-        <v>441</v>
+        <v>452</v>
       </c>
       <c r="E345" t="s">
         <v>155</v>
@@ -41285,7 +41285,7 @@
         <v>1066</v>
       </c>
       <c r="C347" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="D347" t="s">
         <v>54</v>
@@ -42034,7 +42034,7 @@
         <v>1055</v>
       </c>
       <c r="C354" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="D354" t="s">
         <v>200</v>
@@ -43119,7 +43119,7 @@
         <v>151</v>
       </c>
       <c r="H364" t="s">
-        <v>361</v>
+        <v>374</v>
       </c>
       <c r="I364" t="s">
         <v>871</v>
@@ -44896,7 +44896,7 @@
         <v>58</v>
       </c>
       <c r="E2" t="s">
-        <v>131</v>
+        <v>126</v>
       </c>
       <c r="F2" t="s">
         <v>79</v>
@@ -45172,7 +45172,7 @@
         <v>45</v>
       </c>
       <c r="E14" t="s">
-        <v>275</v>
+        <v>293</v>
       </c>
       <c r="F14" t="s">
         <v>79</v>
@@ -45376,7 +45376,7 @@
         <v>1213</v>
       </c>
       <c r="D23" t="s">
-        <v>448</v>
+        <v>438</v>
       </c>
       <c r="E23" t="s">
         <v>1214</v>
@@ -45448,7 +45448,7 @@
         <v>45</v>
       </c>
       <c r="E26" t="s">
-        <v>441</v>
+        <v>452</v>
       </c>
       <c r="F26" t="s">
         <v>366</v>
@@ -45491,7 +45491,7 @@
         <v>1220</v>
       </c>
       <c r="D28" t="s">
-        <v>271</v>
+        <v>289</v>
       </c>
       <c r="E28" t="s">
         <v>43</v>
@@ -45537,7 +45537,7 @@
         <v>1222</v>
       </c>
       <c r="D30" t="s">
-        <v>343</v>
+        <v>360</v>
       </c>
       <c r="E30" t="s">
         <v>79</v>
@@ -45560,7 +45560,7 @@
         <v>1222</v>
       </c>
       <c r="D31" t="s">
-        <v>343</v>
+        <v>360</v>
       </c>
       <c r="E31" t="s">
         <v>79</v>
@@ -45629,7 +45629,7 @@
         <v>1226</v>
       </c>
       <c r="D34" t="s">
-        <v>343</v>
+        <v>360</v>
       </c>
       <c r="E34" t="s">
         <v>45</v>
@@ -45652,7 +45652,7 @@
         <v>1226</v>
       </c>
       <c r="D35" t="s">
-        <v>343</v>
+        <v>360</v>
       </c>
       <c r="E35" t="s">
         <v>45</v>
@@ -45747,7 +45747,7 @@
         <v>45</v>
       </c>
       <c r="E39" t="s">
-        <v>377</v>
+        <v>358</v>
       </c>
       <c r="F39" t="s">
         <v>79</v>

</xml_diff>